<commit_message>
Remove backup scripts and temporary files after data transfer
Co-authored-by: svt.oleksandr <svt.oleksandr@gmail.com>
</commit_message>
<xml_diff>
--- a/Character.edf_main/Class.xlsx
+++ b/Character.edf_main/Class.xlsx
@@ -1003,12 +1003,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Temp</t>
+          <t>KorName</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>KorName</t>
+          <t>EngName</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -1018,27 +1018,27 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>EngName</t>
+          <t>LinkSkill1</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>LinkSkill1</t>
+          <t>LinkSkill2</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>LinkSkill2</t>
+          <t>LinkSkill3</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>LinkSkill3</t>
+          <t>LinkSkill4</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>LinkSkill4</t>
+          <t>LinkSkill5</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>LinkSkill5</t>
+          <t>Reward1</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>Reward1</t>
+          <t>Reward2</t>
         </is>
       </c>
       <c r="CF2" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="CG2" t="inlineStr">
         <is>
-          <t>Reward2</t>
+          <t>Reward3</t>
         </is>
       </c>
       <c r="CH2" t="inlineStr">
@@ -1482,12 +1482,12 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>战士</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Воин</t>
+          <t>WARRIOR</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>WARRIOR</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqbbb00</t>
         </is>
       </c>
       <c r="CD3" t="n">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>iqbbb00</t>
+          <t>ipbhp00</t>
         </is>
       </c>
       <c r="CF3" t="n">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="CG3" t="inlineStr">
         <is>
-          <t>ipbhp00</t>
+          <t>ipbfp00</t>
         </is>
       </c>
       <c r="CH3" t="n">
@@ -1837,12 +1837,12 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>突击队员</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Коммандо</t>
+          <t>COMMANDO</t>
         </is>
       </c>
       <c r="R4" t="n">
@@ -1850,12 +1850,12 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>COMMANDO</t>
+          <t>7F018</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>7F018</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwswb30</t>
         </is>
       </c>
       <c r="CD4" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>iwswb30</t>
+          <t>iwaxb30</t>
         </is>
       </c>
       <c r="CF4" t="n">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="CG4" t="inlineStr">
         <is>
-          <t>iwaxb30</t>
+          <t>iwspb30</t>
         </is>
       </c>
       <c r="CH4" t="n">
@@ -2192,12 +2192,12 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>诱敌者</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Миллер</t>
+          <t>MILER</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -2205,17 +2205,17 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>MILER</t>
+          <t>7F01B</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>7F01B</t>
+          <t>7F01C</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>7F01C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>idbcb29</t>
         </is>
       </c>
       <c r="CD5" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>idbcb29</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF5" t="n">
@@ -2547,12 +2547,12 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>狂武者</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Берсерк</t>
+          <t>BERSERKER</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -2560,27 +2560,27 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>BERSERKER</t>
+          <t>7001E</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>7001E</t>
+          <t>7F01F</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>7F01F</t>
+          <t>7F020</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>7F020</t>
+          <t>7F002</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>7F002</t>
+          <t>70008</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>70008</t>
+          <t>ipbae01</t>
         </is>
       </c>
       <c r="CD6" t="n">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>ipbae01</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF6" t="n">
@@ -2902,12 +2902,12 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>武装者</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Варвар</t>
+          <t>ARMSMAN</t>
         </is>
       </c>
       <c r="R7" t="n">
@@ -2915,27 +2915,27 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>ARMSMAN</t>
+          <t>70021</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>70021</t>
+          <t>7F022</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>7F022</t>
+          <t>7F023</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>7F023</t>
+          <t>7F002</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>7F002</t>
+          <t>70008</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>70008</t>
+          <t>ipbae01</t>
         </is>
       </c>
       <c r="CD7" t="n">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>ipbae01</t>
+          <t>ipbde01</t>
         </is>
       </c>
       <c r="CF7" t="n">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="CG7" t="inlineStr">
         <is>
-          <t>ipbde01</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CH7" t="n">
@@ -3257,12 +3257,12 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>神盾勇者</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Защитник</t>
+          <t>SHIELDMILER</t>
         </is>
       </c>
       <c r="R8" t="n">
@@ -3270,27 +3270,27 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>SHIELDMILER</t>
+          <t>7F024</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>7F024</t>
+          <t>7F025</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>7F025</t>
+          <t>7F026</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>7F026</t>
+          <t>7F002</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>7F002</t>
+          <t>70008</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>70008</t>
+          <t>ipbde01</t>
         </is>
       </c>
       <c r="CD8" t="n">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>ipbde01</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF8" t="n">
@@ -3612,7 +3612,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -3967,7 +3967,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -4322,7 +4322,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -4677,7 +4677,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -5032,7 +5032,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -5387,7 +5387,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -5742,7 +5742,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -6097,7 +6097,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -6452,7 +6452,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>є§¶уЕдАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -6807,12 +6807,12 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>巡察队</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Стрелок</t>
+          <t>RANGER</t>
         </is>
       </c>
       <c r="R18" t="n">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>RANGER</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -7026,7 +7026,7 @@
       </c>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqbbb00</t>
         </is>
       </c>
       <c r="CD18" t="n">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>iqbbb00</t>
+          <t>ipbhp00</t>
         </is>
       </c>
       <c r="CF18" t="n">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="CG18" t="inlineStr">
         <is>
-          <t>ipbhp00</t>
+          <t>ipbfp00</t>
         </is>
       </c>
       <c r="CH18" t="n">
@@ -7162,12 +7162,12 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>暴徒</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Диверсант</t>
+          <t>DESPERADO</t>
         </is>
       </c>
       <c r="R19" t="n">
@@ -7175,12 +7175,12 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>DESPERADO</t>
+          <t>7F096</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>7F096</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="CC19" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwfib30</t>
         </is>
       </c>
       <c r="CD19" t="n">
@@ -7389,7 +7389,7 @@
       </c>
       <c r="CE19" t="inlineStr">
         <is>
-          <t>iwfib30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF19" t="n">
@@ -7517,12 +7517,12 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>狙击手</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Снайпер</t>
+          <t>SNIPER</t>
         </is>
       </c>
       <c r="R20" t="n">
@@ -7530,22 +7530,22 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>SNIPER</t>
+          <t>7F099</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>7F099</t>
+          <t>7F09A</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>7F09A</t>
+          <t>7F09B</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>7F09B</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="CC20" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwbob30</t>
         </is>
       </c>
       <c r="CD20" t="n">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="CE20" t="inlineStr">
         <is>
-          <t>iwbob30</t>
+          <t>tr00001</t>
         </is>
       </c>
       <c r="CF20" t="n">
@@ -7872,12 +7872,12 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>迷踪兵</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Наблюдатель</t>
+          <t>HIDDENSOLDIER</t>
         </is>
       </c>
       <c r="R21" t="n">
@@ -7885,22 +7885,22 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>HIDDENSOLDIER</t>
+          <t>71099</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>71099</t>
+          <t>7F09D</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>7F09D</t>
+          <t>7100C</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>7100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
@@ -8091,7 +8091,7 @@
       </c>
       <c r="CC21" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ibfir34</t>
         </is>
       </c>
       <c r="CD21" t="n">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="CE21" t="inlineStr">
         <is>
-          <t>ibfir34</t>
+          <t>ibfir36</t>
         </is>
       </c>
       <c r="CF21" t="n">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="CG21" t="inlineStr">
         <is>
-          <t>ibfir36</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CH21" t="n">
@@ -8227,12 +8227,12 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>禁卫军</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Страж</t>
+          <t>SENTINEL</t>
         </is>
       </c>
       <c r="R22" t="n">
@@ -8240,27 +8240,27 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>SENTINEL</t>
+          <t>7F09F</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>7F09F</t>
+          <t>7F0A0</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>7F0A0</t>
+          <t>7F0A1</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>7F0A1</t>
+          <t>7100C</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>7100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -8446,7 +8446,7 @@
       </c>
       <c r="CC22" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ibbow48</t>
         </is>
       </c>
       <c r="CD22" t="n">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="CE22" t="inlineStr">
         <is>
-          <t>ibbow48</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF22" t="n">
@@ -8582,12 +8582,12 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>渗透者</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Шпион</t>
+          <t>INFILTRATOR</t>
         </is>
       </c>
       <c r="R23" t="n">
@@ -8595,22 +8595,22 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>INFILTRATOR</t>
+          <t>700A2</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>700A2</t>
+          <t>7F0A3</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>7F0A3</t>
+          <t>7100C</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>7100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -8801,7 +8801,7 @@
       </c>
       <c r="CC23" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwdka40</t>
         </is>
       </c>
       <c r="CD23" t="n">
@@ -8809,7 +8809,7 @@
       </c>
       <c r="CE23" t="inlineStr">
         <is>
-          <t>iwdka40</t>
+          <t>tr00002</t>
         </is>
       </c>
       <c r="CF23" t="n">
@@ -8937,7 +8937,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -9292,7 +9292,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -9647,7 +9647,7 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -10002,7 +10002,7 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -10357,7 +10357,7 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -10712,7 +10712,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -11067,7 +11067,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -11422,7 +11422,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -11777,7 +11777,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>є§¶уЕд·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -12132,12 +12132,12 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>神灵使者</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Колдун</t>
+          <t>SPIRITUALIST</t>
         </is>
       </c>
       <c r="R33" t="n">
@@ -12145,7 +12145,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>SPIRITUALIST</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="CC33" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqbbb00</t>
         </is>
       </c>
       <c r="CD33" t="n">
@@ -12359,7 +12359,7 @@
       </c>
       <c r="CE33" t="inlineStr">
         <is>
-          <t>iqbbb00</t>
+          <t>ipbhp00</t>
         </is>
       </c>
       <c r="CF33" t="n">
@@ -12367,7 +12367,7 @@
       </c>
       <c r="CG33" t="inlineStr">
         <is>
-          <t>ipbhp00</t>
+          <t>ipbfp00</t>
         </is>
       </c>
       <c r="CH33" t="n">
@@ -12487,12 +12487,12 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>操灵师</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Псионик</t>
+          <t>PSYPER</t>
         </is>
       </c>
       <c r="R34" t="n">
@@ -12500,12 +12500,12 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>PSYPER</t>
+          <t>7F114</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>7F114</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -12706,7 +12706,7 @@
       </c>
       <c r="CC34" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwstb30</t>
         </is>
       </c>
       <c r="CD34" t="n">
@@ -12714,7 +12714,7 @@
       </c>
       <c r="CE34" t="inlineStr">
         <is>
-          <t>iwstb30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF34" t="n">
@@ -12842,12 +12842,12 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>斩德拉</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Чародей</t>
+          <t>CANDRA</t>
         </is>
       </c>
       <c r="R35" t="n">
@@ -12855,17 +12855,17 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>CANDRA</t>
+          <t>7F117</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>7F117</t>
+          <t>7F118</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>7F118</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -13061,7 +13061,7 @@
       </c>
       <c r="CC35" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwstb30</t>
         </is>
       </c>
       <c r="CD35" t="n">
@@ -13069,7 +13069,7 @@
       </c>
       <c r="CE35" t="inlineStr">
         <is>
-          <t>iwstb30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF35" t="n">
@@ -13197,12 +13197,12 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>巫师</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Волшебник</t>
+          <t>WIZARD</t>
         </is>
       </c>
       <c r="R36" t="n">
@@ -13210,22 +13210,22 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>WIZARD</t>
+          <t>7F11A</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>7F11A</t>
+          <t>7011B</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>7011B</t>
+          <t>7111C</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>7111C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
@@ -13416,7 +13416,7 @@
       </c>
       <c r="CC36" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>icfha01</t>
         </is>
       </c>
       <c r="CD36" t="n">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="CE36" t="inlineStr">
         <is>
-          <t>icfha01</t>
+          <t>icfha02</t>
         </is>
       </c>
       <c r="CF36" t="n">
@@ -13432,7 +13432,7 @@
       </c>
       <c r="CG36" t="inlineStr">
         <is>
-          <t>icfha02</t>
+          <t>icfha03</t>
         </is>
       </c>
       <c r="CH36" t="n">
@@ -13552,12 +13552,12 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>灵魂使</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Медиум</t>
+          <t>ASTRAL</t>
         </is>
       </c>
       <c r="R37" t="n">
@@ -13565,22 +13565,22 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>ASTRAL</t>
+          <t>7F11D</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>7F11D</t>
+          <t>7F11E</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>7F11E</t>
+          <t>7F11F</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>7F11F</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
@@ -13771,7 +13771,7 @@
       </c>
       <c r="CC37" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>icaha03</t>
         </is>
       </c>
       <c r="CD37" t="n">
@@ -13779,7 +13779,7 @@
       </c>
       <c r="CE37" t="inlineStr">
         <is>
-          <t>icaha03</t>
+          <t>icaha04</t>
         </is>
       </c>
       <c r="CF37" t="n">
@@ -13787,7 +13787,7 @@
       </c>
       <c r="CG37" t="inlineStr">
         <is>
-          <t>icaha04</t>
+          <t>ictha03</t>
         </is>
       </c>
       <c r="CH37" t="n">
@@ -13907,12 +13907,12 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>神圣斩德拉</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Чудотворец</t>
+          <t>HOLYCANDRA</t>
         </is>
       </c>
       <c r="R38" t="n">
@@ -13920,22 +13920,22 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>HOLYCANDRA</t>
+          <t>7F120</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>7F120</t>
+          <t>7F121</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>7F121</t>
+          <t>7F122</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>7F122</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
@@ -14126,7 +14126,7 @@
       </c>
       <c r="CC38" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ichhs01</t>
         </is>
       </c>
       <c r="CD38" t="n">
@@ -14134,7 +14134,7 @@
       </c>
       <c r="CE38" t="inlineStr">
         <is>
-          <t>ichhs01</t>
+          <t>ichhs02</t>
         </is>
       </c>
       <c r="CF38" t="n">
@@ -14142,7 +14142,7 @@
       </c>
       <c r="CG38" t="inlineStr">
         <is>
-          <t>ichhs02</t>
+          <t>ichhs03</t>
         </is>
       </c>
       <c r="CH38" t="n">
@@ -14262,7 +14262,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -14617,7 +14617,7 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -14972,7 +14972,7 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -15327,7 +15327,7 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -15682,7 +15682,7 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -16037,7 +16037,7 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -16392,7 +16392,7 @@
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -16747,7 +16747,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -17102,7 +17102,7 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>є§¶уЕдБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -17457,12 +17457,12 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>专家</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>Специалист</t>
+          <t>SPECIALIST</t>
         </is>
       </c>
       <c r="R48" t="n">
@@ -17470,7 +17470,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>SPECIALIST</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -17676,7 +17676,7 @@
       </c>
       <c r="CC48" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqbbb00</t>
         </is>
       </c>
       <c r="CD48" t="n">
@@ -17684,7 +17684,7 @@
       </c>
       <c r="CE48" t="inlineStr">
         <is>
-          <t>iqbbb00</t>
+          <t>iwmtb00</t>
         </is>
       </c>
       <c r="CF48" t="n">
@@ -17692,7 +17692,7 @@
       </c>
       <c r="CG48" t="inlineStr">
         <is>
-          <t>iwmtb00</t>
+          <t>itttt00</t>
         </is>
       </c>
       <c r="CH48" t="n">
@@ -17812,12 +17812,12 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>匠师</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Ремесленник</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="R49" t="n">
@@ -17825,12 +17825,12 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>7F192</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>7F192</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -18031,7 +18031,7 @@
       </c>
       <c r="CC49" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>gtbb001</t>
         </is>
       </c>
       <c r="CD49" t="n">
@@ -18167,12 +18167,12 @@
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>战斗驾驶</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Пилот</t>
+          <t>DRIVER</t>
         </is>
       </c>
       <c r="R50" t="n">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -18386,7 +18386,7 @@
       </c>
       <c r="CC50" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwbob30</t>
         </is>
       </c>
       <c r="CD50" t="n">
@@ -18394,7 +18394,7 @@
       </c>
       <c r="CE50" t="inlineStr">
         <is>
-          <t>iwbob30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF50" t="n">
@@ -18522,12 +18522,12 @@
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>睿智工匠</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Кузнец</t>
+          <t>MENTALSMITH</t>
         </is>
       </c>
       <c r="R51" t="n">
@@ -18535,17 +18535,17 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>MENTALSMITH</t>
+          <t>7F198</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>7F198</t>
+          <t>7F199</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>7F199</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">
@@ -18741,7 +18741,7 @@
       </c>
       <c r="CC51" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iaxxx09</t>
         </is>
       </c>
       <c r="CD51" t="n">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="CE51" t="inlineStr">
         <is>
-          <t>iaxxx09</t>
+          <t>irgef03</t>
         </is>
       </c>
       <c r="CF51" t="n">
@@ -18757,7 +18757,7 @@
       </c>
       <c r="CG51" t="inlineStr">
         <is>
-          <t>irgef03</t>
+          <t>irgea03</t>
         </is>
       </c>
       <c r="CH51" t="n">
@@ -18877,12 +18877,12 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>武装驾驶</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Технорыцарь</t>
+          <t>ARMORRIDER</t>
         </is>
       </c>
       <c r="R52" t="n">
@@ -18890,17 +18890,17 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>ARMORRIDER</t>
+          <t>7F19B</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>7F19B</t>
+          <t>7F19C</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>7F19C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
@@ -19096,7 +19096,7 @@
       </c>
       <c r="CC52" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iaxxx09</t>
         </is>
       </c>
       <c r="CD52" t="n">
@@ -19104,7 +19104,7 @@
       </c>
       <c r="CE52" t="inlineStr">
         <is>
-          <t>iaxxx09</t>
+          <t>irgef03</t>
         </is>
       </c>
       <c r="CF52" t="n">
@@ -19112,7 +19112,7 @@
       </c>
       <c r="CG52" t="inlineStr">
         <is>
-          <t>irgef03</t>
+          <t>irgea03</t>
         </is>
       </c>
       <c r="CH52" t="n">
@@ -19232,7 +19232,7 @@
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -19587,7 +19587,7 @@
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -19942,7 +19942,7 @@
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -20297,7 +20297,7 @@
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -20652,7 +20652,7 @@
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -21007,7 +21007,7 @@
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -21362,7 +21362,7 @@
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -21717,7 +21717,7 @@
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -22072,7 +22072,7 @@
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -22427,7 +22427,7 @@
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>є§¶уЕдЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -22782,12 +22782,12 @@
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>战士</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Воин</t>
+          <t>WARRIOR</t>
         </is>
       </c>
       <c r="R63" t="n">
@@ -22795,7 +22795,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>WARRIOR</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
@@ -23001,7 +23001,7 @@
       </c>
       <c r="CC63" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqccc00</t>
         </is>
       </c>
       <c r="CD63" t="n">
@@ -23009,7 +23009,7 @@
       </c>
       <c r="CE63" t="inlineStr">
         <is>
-          <t>iqccc00</t>
+          <t>ipchp00</t>
         </is>
       </c>
       <c r="CF63" t="n">
@@ -23017,7 +23017,7 @@
       </c>
       <c r="CG63" t="inlineStr">
         <is>
-          <t>ipchp00</t>
+          <t>ipcfp00</t>
         </is>
       </c>
       <c r="CH63" t="n">
@@ -23137,12 +23137,12 @@
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>斗士</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Чемпион</t>
+          <t>CHAMPION</t>
         </is>
       </c>
       <c r="R64" t="n">
@@ -23150,17 +23150,17 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>CHAMPION</t>
+          <t>8F042</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>8F042</t>
+          <t>8F043</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>8F043</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V64" t="inlineStr">
@@ -23356,7 +23356,7 @@
       </c>
       <c r="CC64" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwswb30</t>
         </is>
       </c>
       <c r="CD64" t="n">
@@ -23364,7 +23364,7 @@
       </c>
       <c r="CE64" t="inlineStr">
         <is>
-          <t>iwswb30</t>
+          <t>iwaxb30</t>
         </is>
       </c>
       <c r="CF64" t="n">
@@ -23372,7 +23372,7 @@
       </c>
       <c r="CG64" t="inlineStr">
         <is>
-          <t>iwaxb30</t>
+          <t>iwspb30</t>
         </is>
       </c>
       <c r="CH64" t="n">
@@ -23492,12 +23492,12 @@
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>骑兵</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Рыцарь</t>
+          <t>KNIGHTS</t>
         </is>
       </c>
       <c r="R65" t="n">
@@ -23505,22 +23505,22 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>KNIGHTS</t>
+          <t>8F045</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
         <is>
-          <t>8F045</t>
+          <t>8F046</t>
         </is>
       </c>
       <c r="U65" t="inlineStr">
         <is>
-          <t>8F046</t>
+          <t>8F047</t>
         </is>
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>8F047</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W65" t="inlineStr">
@@ -23711,7 +23711,7 @@
       </c>
       <c r="CC65" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>idbcb29</t>
         </is>
       </c>
       <c r="CD65" t="n">
@@ -23719,7 +23719,7 @@
       </c>
       <c r="CE65" t="inlineStr">
         <is>
-          <t>idbcb29</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF65" t="n">
@@ -23847,12 +23847,12 @@
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>圣殿骑士</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Храмовник</t>
+          <t>TEMPLAR</t>
         </is>
       </c>
       <c r="R66" t="n">
@@ -23860,27 +23860,27 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>TEMPLAR</t>
+          <t>80048</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>80048</t>
+          <t>8F049</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
         <is>
-          <t>8F049</t>
+          <t>8F04A</t>
         </is>
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>8F04A</t>
+          <t>8F002</t>
         </is>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>8F002</t>
+          <t>80008</t>
         </is>
       </c>
       <c r="X66" t="inlineStr">
@@ -24066,7 +24066,7 @@
       </c>
       <c r="CC66" t="inlineStr">
         <is>
-          <t>80008</t>
+          <t>ipbae02</t>
         </is>
       </c>
       <c r="CD66" t="n">
@@ -24074,7 +24074,7 @@
       </c>
       <c r="CE66" t="inlineStr">
         <is>
-          <t>ipbae02</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF66" t="n">
@@ -24202,12 +24202,12 @@
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>审判骑士</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>Хранитель</t>
+          <t>GUARDIAN</t>
         </is>
       </c>
       <c r="R67" t="n">
@@ -24215,27 +24215,27 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>GUARDIAN</t>
+          <t>8F04B</t>
         </is>
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>8F04B</t>
+          <t>8F04C</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>8F04C</t>
+          <t>8F002</t>
         </is>
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>8F002</t>
+          <t>80008</t>
         </is>
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>80008</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X67" t="inlineStr">
@@ -24421,7 +24421,7 @@
       </c>
       <c r="CC67" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ipbae02</t>
         </is>
       </c>
       <c r="CD67" t="n">
@@ -24429,7 +24429,7 @@
       </c>
       <c r="CE67" t="inlineStr">
         <is>
-          <t>ipbae02</t>
+          <t>ipbde02</t>
         </is>
       </c>
       <c r="CF67" t="n">
@@ -24437,7 +24437,7 @@
       </c>
       <c r="CG67" t="inlineStr">
         <is>
-          <t>ipbde02</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CH67" t="n">
@@ -24557,12 +24557,12 @@
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>黑暗骑士</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>Черный рыцарь</t>
+          <t>BLACKKNIGHTS</t>
         </is>
       </c>
       <c r="R68" t="n">
@@ -24570,27 +24570,27 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>BLACKKNIGHTS</t>
+          <t>8F04E</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
         <is>
-          <t>8F04E</t>
+          <t>8F04F</t>
         </is>
       </c>
       <c r="U68" t="inlineStr">
         <is>
-          <t>8F04F</t>
+          <t>8F002</t>
         </is>
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>8F002</t>
+          <t>80008</t>
         </is>
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>80008</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X68" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="CC68" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ipbde02</t>
         </is>
       </c>
       <c r="CD68" t="n">
@@ -24784,7 +24784,7 @@
       </c>
       <c r="CE68" t="inlineStr">
         <is>
-          <t>ipbde02</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF68" t="n">
@@ -24912,7 +24912,7 @@
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -25267,7 +25267,7 @@
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -25622,7 +25622,7 @@
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -25977,7 +25977,7 @@
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
@@ -26332,7 +26332,7 @@
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -26687,7 +26687,7 @@
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -27042,7 +27042,7 @@
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -27397,7 +27397,7 @@
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -27752,7 +27752,7 @@
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
-          <t>ДЪ¶уАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -28107,12 +28107,12 @@
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>巡察队</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>Стрелок</t>
+          <t>RANGER</t>
         </is>
       </c>
       <c r="R78" t="n">
@@ -28120,7 +28120,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>RANGER</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="CC78" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqccc00</t>
         </is>
       </c>
       <c r="CD78" t="n">
@@ -28334,7 +28334,7 @@
       </c>
       <c r="CE78" t="inlineStr">
         <is>
-          <t>iqccc00</t>
+          <t>ipchp00</t>
         </is>
       </c>
       <c r="CF78" t="n">
@@ -28342,7 +28342,7 @@
       </c>
       <c r="CG78" t="inlineStr">
         <is>
-          <t>ipchp00</t>
+          <t>ipcfp00</t>
         </is>
       </c>
       <c r="CH78" t="n">
@@ -28462,12 +28462,12 @@
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>弓箭手</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>Лучник</t>
+          <t>ARCHER</t>
         </is>
       </c>
       <c r="R79" t="n">
@@ -28475,17 +28475,17 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>ARCHER</t>
+          <t>8F0C0</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
         <is>
-          <t>8F0C0</t>
+          <t>810C1</t>
         </is>
       </c>
       <c r="U79" t="inlineStr">
         <is>
-          <t>810C1</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V79" t="inlineStr">
@@ -28681,7 +28681,7 @@
       </c>
       <c r="CC79" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwbob30</t>
         </is>
       </c>
       <c r="CD79" t="n">
@@ -28689,7 +28689,7 @@
       </c>
       <c r="CE79" t="inlineStr">
         <is>
-          <t>iwbob30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF79" t="n">
@@ -28817,12 +28817,12 @@
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>猎杀者</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>Охотник</t>
+          <t>HUNTER</t>
         </is>
       </c>
       <c r="R80" t="n">
@@ -28830,22 +28830,22 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>HUNTER</t>
+          <t>8F0C3</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
         <is>
-          <t>8F0C3</t>
+          <t>8F0C4</t>
         </is>
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>8F0C4</t>
+          <t>8F0C5</t>
         </is>
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>8F0C5</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W80" t="inlineStr">
@@ -29036,7 +29036,7 @@
       </c>
       <c r="CC80" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwfib30</t>
         </is>
       </c>
       <c r="CD80" t="n">
@@ -29044,7 +29044,7 @@
       </c>
       <c r="CE80" t="inlineStr">
         <is>
-          <t>iwfib30</t>
+          <t>tr00001</t>
         </is>
       </c>
       <c r="CF80" t="n">
@@ -29172,12 +29172,12 @@
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>冒险者</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>Наемник</t>
+          <t>ADVENTURER</t>
         </is>
       </c>
       <c r="R81" t="n">
@@ -29185,22 +29185,22 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>ADVENTURER</t>
+          <t>8F0C6</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
         <is>
-          <t>8F0C6</t>
+          <t>8F0C7</t>
         </is>
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>8F0C7</t>
+          <t>8100C</t>
         </is>
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>8100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W81" t="inlineStr">
@@ -29391,7 +29391,7 @@
       </c>
       <c r="CC81" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ibbow48</t>
         </is>
       </c>
       <c r="CD81" t="n">
@@ -29399,7 +29399,7 @@
       </c>
       <c r="CE81" t="inlineStr">
         <is>
-          <t>ibbow48</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF81" t="n">
@@ -29527,12 +29527,12 @@
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>异端杀手</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>Отступник</t>
+          <t>STEELER</t>
         </is>
       </c>
       <c r="R82" t="n">
@@ -29540,27 +29540,27 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>STEELER</t>
+          <t>8F0C9</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
         <is>
-          <t>8F0C9</t>
+          <t>8F0CA</t>
         </is>
       </c>
       <c r="U82" t="inlineStr">
         <is>
-          <t>8F0CA</t>
+          <t>8F0CB</t>
         </is>
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>8F0CB</t>
+          <t>8100C</t>
         </is>
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>8100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X82" t="inlineStr">
@@ -29746,7 +29746,7 @@
       </c>
       <c r="CC82" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ibfir34</t>
         </is>
       </c>
       <c r="CD82" t="n">
@@ -29754,7 +29754,7 @@
       </c>
       <c r="CE82" t="inlineStr">
         <is>
-          <t>ibfir34</t>
+          <t>ibfir36</t>
         </is>
       </c>
       <c r="CF82" t="n">
@@ -29762,7 +29762,7 @@
       </c>
       <c r="CG82" t="inlineStr">
         <is>
-          <t>ibfir36</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CH82" t="n">
@@ -29882,12 +29882,12 @@
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>暗杀者</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Ассасин</t>
+          <t>ASSASSIN</t>
         </is>
       </c>
       <c r="R83" t="n">
@@ -29895,22 +29895,22 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>ASSASSIN</t>
+          <t>800CC</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
         <is>
-          <t>800CC</t>
+          <t>8F0CD</t>
         </is>
       </c>
       <c r="U83" t="inlineStr">
         <is>
-          <t>8F0CD</t>
+          <t>8100C</t>
         </is>
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>8100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W83" t="inlineStr">
@@ -30101,7 +30101,7 @@
       </c>
       <c r="CC83" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwdka40</t>
         </is>
       </c>
       <c r="CD83" t="n">
@@ -30109,7 +30109,7 @@
       </c>
       <c r="CE83" t="inlineStr">
         <is>
-          <t>iwdka40</t>
+          <t>tr00002</t>
         </is>
       </c>
       <c r="CF83" t="n">
@@ -30237,7 +30237,7 @@
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
@@ -30592,7 +30592,7 @@
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -30947,7 +30947,7 @@
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -31302,7 +31302,7 @@
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -31657,7 +31657,7 @@
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
@@ -32012,7 +32012,7 @@
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -32367,7 +32367,7 @@
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -32722,7 +32722,7 @@
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -33077,7 +33077,7 @@
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr">
         <is>
-          <t>ДЪ¶у·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
@@ -33432,12 +33432,12 @@
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>神灵使者</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>Колдун</t>
+          <t>SPIRITUALIST</t>
         </is>
       </c>
       <c r="R93" t="n">
@@ -33445,7 +33445,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>SPIRITUALIST</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T93" t="inlineStr">
@@ -33651,7 +33651,7 @@
       </c>
       <c r="CC93" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqccc00</t>
         </is>
       </c>
       <c r="CD93" t="n">
@@ -33659,7 +33659,7 @@
       </c>
       <c r="CE93" t="inlineStr">
         <is>
-          <t>iqccc00</t>
+          <t>ipchp00</t>
         </is>
       </c>
       <c r="CF93" t="n">
@@ -33667,7 +33667,7 @@
       </c>
       <c r="CG93" t="inlineStr">
         <is>
-          <t>ipchp00</t>
+          <t>ipcfp00</t>
         </is>
       </c>
       <c r="CH93" t="n">
@@ -33787,12 +33787,12 @@
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>暗灵使</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Маг</t>
+          <t>CASTER</t>
         </is>
       </c>
       <c r="R94" t="n">
@@ -33800,12 +33800,12 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>CASTER</t>
+          <t>8F13E</t>
         </is>
       </c>
       <c r="T94" t="inlineStr">
         <is>
-          <t>8F13E</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U94" t="inlineStr">
@@ -34006,7 +34006,7 @@
       </c>
       <c r="CC94" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwstb30</t>
         </is>
       </c>
       <c r="CD94" t="n">
@@ -34014,7 +34014,7 @@
       </c>
       <c r="CE94" t="inlineStr">
         <is>
-          <t>iwstb30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF94" t="n">
@@ -34142,12 +34142,12 @@
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>召唤师</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Вызыватель</t>
+          <t>SUMMONER</t>
         </is>
       </c>
       <c r="R95" t="n">
@@ -34155,7 +34155,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>SUMMONER</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T95" t="inlineStr">
@@ -34361,7 +34361,7 @@
       </c>
       <c r="CC95" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ijccc01</t>
         </is>
       </c>
       <c r="CD95" t="n">
@@ -34369,7 +34369,7 @@
       </c>
       <c r="CE95" t="inlineStr">
         <is>
-          <t>ijccc01</t>
+          <t>ijccc02</t>
         </is>
       </c>
       <c r="CF95" t="n">
@@ -34377,7 +34377,7 @@
       </c>
       <c r="CG95" t="inlineStr">
         <is>
-          <t>ijccc02</t>
+          <t>ijccc03</t>
         </is>
       </c>
       <c r="CH95" t="n">
@@ -34497,12 +34497,12 @@
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>魔咒师</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>Чернокнижник</t>
+          <t>WARLOCK</t>
         </is>
       </c>
       <c r="R96" t="n">
@@ -34510,22 +34510,22 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>WARLOCK</t>
+          <t>8F144</t>
         </is>
       </c>
       <c r="T96" t="inlineStr">
         <is>
-          <t>8F144</t>
+          <t>8F145</t>
         </is>
       </c>
       <c r="U96" t="inlineStr">
         <is>
-          <t>8F145</t>
+          <t>81146</t>
         </is>
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>81146</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W96" t="inlineStr">
@@ -34716,7 +34716,7 @@
       </c>
       <c r="CC96" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>icfha01</t>
         </is>
       </c>
       <c r="CD96" t="n">
@@ -34724,7 +34724,7 @@
       </c>
       <c r="CE96" t="inlineStr">
         <is>
-          <t>icfha01</t>
+          <t>icfha02</t>
         </is>
       </c>
       <c r="CF96" t="n">
@@ -34732,7 +34732,7 @@
       </c>
       <c r="CG96" t="inlineStr">
         <is>
-          <t>icfha02</t>
+          <t>icfha03</t>
         </is>
       </c>
       <c r="CH96" t="n">
@@ -34852,12 +34852,12 @@
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>暗灵祭司</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>Темный жрец</t>
+          <t>DARKPRIEST</t>
         </is>
       </c>
       <c r="R97" t="n">
@@ -34865,22 +34865,22 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>DARKPRIEST</t>
+          <t>8F147</t>
         </is>
       </c>
       <c r="T97" t="inlineStr">
         <is>
-          <t>8F147</t>
+          <t>8F148</t>
         </is>
       </c>
       <c r="U97" t="inlineStr">
         <is>
-          <t>8F148</t>
+          <t>8F149</t>
         </is>
       </c>
       <c r="V97" t="inlineStr">
         <is>
-          <t>8F149</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W97" t="inlineStr">
@@ -35071,7 +35071,7 @@
       </c>
       <c r="CC97" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>icaha03</t>
         </is>
       </c>
       <c r="CD97" t="n">
@@ -35079,7 +35079,7 @@
       </c>
       <c r="CE97" t="inlineStr">
         <is>
-          <t>icaha03</t>
+          <t>icaha04</t>
         </is>
       </c>
       <c r="CF97" t="n">
@@ -35087,7 +35087,7 @@
       </c>
       <c r="CG97" t="inlineStr">
         <is>
-          <t>icaha04</t>
+          <t>ictha03</t>
         </is>
       </c>
       <c r="CH97" t="n">
@@ -35207,12 +35207,12 @@
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>幻兽牧者</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>Пастырь</t>
+          <t>GRAZIER</t>
         </is>
       </c>
       <c r="R98" t="n">
@@ -35220,27 +35220,27 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>GRAZIER</t>
+          <t>8F14A</t>
         </is>
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>8F14A</t>
+          <t>8F14B</t>
         </is>
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>8F14B</t>
+          <t>8F14C</t>
         </is>
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>8F14C</t>
+          <t>8F14D</t>
         </is>
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>8F14D</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X98" t="inlineStr">
@@ -35426,7 +35426,7 @@
       </c>
       <c r="CC98" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ijccc04</t>
         </is>
       </c>
       <c r="CD98" t="n">
@@ -35434,7 +35434,7 @@
       </c>
       <c r="CE98" t="inlineStr">
         <is>
-          <t>ijccc04</t>
+          <t>icdhs01</t>
         </is>
       </c>
       <c r="CF98" t="n">
@@ -35442,7 +35442,7 @@
       </c>
       <c r="CG98" t="inlineStr">
         <is>
-          <t>icdhs01</t>
+          <t>icdhs02</t>
         </is>
       </c>
       <c r="CH98" t="n">
@@ -35562,7 +35562,7 @@
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
@@ -35917,7 +35917,7 @@
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -36272,7 +36272,7 @@
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -36627,7 +36627,7 @@
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -36982,7 +36982,7 @@
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -37337,7 +37337,7 @@
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -37692,7 +37692,7 @@
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -38047,7 +38047,7 @@
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -38402,7 +38402,7 @@
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr">
         <is>
-          <t>ДЪ¶уБ¤ЅЕ°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -38757,12 +38757,12 @@
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>专家</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>Специалист</t>
+          <t>SPECIALIST</t>
         </is>
       </c>
       <c r="R108" t="n">
@@ -38770,7 +38770,7 @@
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>SPECIALIST</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T108" t="inlineStr">
@@ -38976,7 +38976,7 @@
       </c>
       <c r="CC108" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqccc00</t>
         </is>
       </c>
       <c r="CD108" t="n">
@@ -38984,7 +38984,7 @@
       </c>
       <c r="CE108" t="inlineStr">
         <is>
-          <t>iqccc00</t>
+          <t>iwmtc00</t>
         </is>
       </c>
       <c r="CF108" t="n">
@@ -38992,7 +38992,7 @@
       </c>
       <c r="CG108" t="inlineStr">
         <is>
-          <t>iwmtc00</t>
+          <t>itttt00</t>
         </is>
       </c>
       <c r="CH108" t="n">
@@ -39112,12 +39112,12 @@
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>匠师</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>Ремесленник</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="R109" t="n">
@@ -39125,12 +39125,12 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>8F1BC</t>
         </is>
       </c>
       <c r="T109" t="inlineStr">
         <is>
-          <t>8F1BC</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U109" t="inlineStr">
@@ -39331,7 +39331,7 @@
       </c>
       <c r="CC109" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>gtcc001</t>
         </is>
       </c>
       <c r="CD109" t="n">
@@ -39467,7 +39467,7 @@
       <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -39822,12 +39822,12 @@
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>天艺匠师</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>Артизан</t>
+          <t>ARTIST</t>
         </is>
       </c>
       <c r="R111" t="n">
@@ -39835,17 +39835,17 @@
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>ARTIST</t>
+          <t>8F1C2</t>
         </is>
       </c>
       <c r="T111" t="inlineStr">
         <is>
-          <t>8F1C2</t>
+          <t>8F1C3</t>
         </is>
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>8F1C3</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V111" t="inlineStr">
@@ -40041,7 +40041,7 @@
       </c>
       <c r="CC111" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iaxxx09</t>
         </is>
       </c>
       <c r="CD111" t="n">
@@ -40049,7 +40049,7 @@
       </c>
       <c r="CE111" t="inlineStr">
         <is>
-          <t>iaxxx09</t>
+          <t>irgef03</t>
         </is>
       </c>
       <c r="CF111" t="n">
@@ -40057,7 +40057,7 @@
       </c>
       <c r="CG111" t="inlineStr">
         <is>
-          <t>irgef03</t>
+          <t>irgea03</t>
         </is>
       </c>
       <c r="CH111" t="n">
@@ -40177,7 +40177,7 @@
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -40532,7 +40532,7 @@
       <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
@@ -40887,7 +40887,7 @@
       <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -41242,7 +41242,7 @@
       <c r="O115" t="inlineStr"/>
       <c r="P115" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -41597,7 +41597,7 @@
       <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
@@ -41952,7 +41952,7 @@
       <c r="O117" t="inlineStr"/>
       <c r="P117" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr">
@@ -42307,7 +42307,7 @@
       <c r="O118" t="inlineStr"/>
       <c r="P118" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr">
@@ -42662,7 +42662,7 @@
       <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -43017,7 +43017,7 @@
       <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -43372,7 +43372,7 @@
       <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -43727,7 +43727,7 @@
       <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr">
         <is>
-          <t>ДЪ¶уЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
@@ -44082,12 +44082,12 @@
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>战士</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>Воин</t>
+          <t>WARRIOR</t>
         </is>
       </c>
       <c r="R123" t="n">
@@ -44095,7 +44095,7 @@
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>WARRIOR</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T123" t="inlineStr">
@@ -44301,7 +44301,7 @@
       </c>
       <c r="CC123" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqaaa00</t>
         </is>
       </c>
       <c r="CD123" t="n">
@@ -44309,7 +44309,7 @@
       </c>
       <c r="CE123" t="inlineStr">
         <is>
-          <t>iqaaa00</t>
+          <t>ipahp00</t>
         </is>
       </c>
       <c r="CF123" t="n">
@@ -44317,7 +44317,7 @@
       </c>
       <c r="CG123" t="inlineStr">
         <is>
-          <t>ipahp00</t>
+          <t>ipafp00</t>
         </is>
       </c>
       <c r="CH123" t="n">
@@ -44437,12 +44437,12 @@
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>毁灭者</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>Разрушитель</t>
+          <t>DESTROYER</t>
         </is>
       </c>
       <c r="R124" t="n">
@@ -44450,17 +44450,17 @@
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>DESTROYER</t>
+          <t>4006C</t>
         </is>
       </c>
       <c r="T124" t="inlineStr">
         <is>
-          <t>4006C</t>
+          <t>4F06D</t>
         </is>
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>4F06D</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V124" t="inlineStr">
@@ -44656,7 +44656,7 @@
       </c>
       <c r="CC124" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwswb30</t>
         </is>
       </c>
       <c r="CD124" t="n">
@@ -44664,7 +44664,7 @@
       </c>
       <c r="CE124" t="inlineStr">
         <is>
-          <t>iwswb30</t>
+          <t>iwaxb30</t>
         </is>
       </c>
       <c r="CF124" t="n">
@@ -44672,7 +44672,7 @@
       </c>
       <c r="CG124" t="inlineStr">
         <is>
-          <t>iwaxb30</t>
+          <t>iwspb30</t>
         </is>
       </c>
       <c r="CH124" t="n">
@@ -44792,12 +44792,12 @@
       <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>神鬼战士</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>Гладиатор</t>
+          <t>GLADIUS</t>
         </is>
       </c>
       <c r="R125" t="n">
@@ -44805,22 +44805,22 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>GLADIUS</t>
+          <t>4F06F</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
         <is>
-          <t>4F06F</t>
+          <t>4F070</t>
         </is>
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>4F070</t>
+          <t>4F071</t>
         </is>
       </c>
       <c r="V125" t="inlineStr">
         <is>
-          <t>4F071</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W125" t="inlineStr">
@@ -45011,7 +45011,7 @@
       </c>
       <c r="CC125" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>idaab29</t>
         </is>
       </c>
       <c r="CD125" t="n">
@@ -45019,7 +45019,7 @@
       </c>
       <c r="CE125" t="inlineStr">
         <is>
-          <t>idaab29</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF125" t="n">
@@ -45147,12 +45147,12 @@
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>制裁者</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Каратель</t>
+          <t>PUNISHER</t>
         </is>
       </c>
       <c r="R126" t="n">
@@ -45160,27 +45160,27 @@
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>PUNISHER</t>
+          <t>4F072</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
         <is>
-          <t>4F072</t>
+          <t>4F073</t>
         </is>
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>4F073</t>
+          <t>4F074</t>
         </is>
       </c>
       <c r="V126" t="inlineStr">
         <is>
-          <t>4F074</t>
+          <t>4F002</t>
         </is>
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>4F002</t>
+          <t>40008</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -45366,7 +45366,7 @@
       </c>
       <c r="CC126" t="inlineStr">
         <is>
-          <t>40008</t>
+          <t>ipbae03</t>
         </is>
       </c>
       <c r="CD126" t="n">
@@ -45374,7 +45374,7 @@
       </c>
       <c r="CE126" t="inlineStr">
         <is>
-          <t>ipbae03</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF126" t="n">
@@ -45502,12 +45502,12 @@
       <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>强袭战士</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>Штурмовик</t>
+          <t>ASSAULTER</t>
         </is>
       </c>
       <c r="R127" t="n">
@@ -45515,27 +45515,27 @@
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>ASSAULTER</t>
+          <t>4F075</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
         <is>
-          <t>4F075</t>
+          <t>4F076</t>
         </is>
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>4F076</t>
+          <t>4F002</t>
         </is>
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>4F002</t>
+          <t>40008</t>
         </is>
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>40008</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
@@ -45721,7 +45721,7 @@
       </c>
       <c r="CC127" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ipbae03</t>
         </is>
       </c>
       <c r="CD127" t="n">
@@ -45729,7 +45729,7 @@
       </c>
       <c r="CE127" t="inlineStr">
         <is>
-          <t>ipbae03</t>
+          <t>ipbde03</t>
         </is>
       </c>
       <c r="CF127" t="n">
@@ -45737,7 +45737,7 @@
       </c>
       <c r="CG127" t="inlineStr">
         <is>
-          <t>ipbde03</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CH127" t="n">
@@ -45857,12 +45857,12 @@
       <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>超能战士</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>Ландскнехт</t>
+          <t>MERCENARY</t>
         </is>
       </c>
       <c r="R128" t="n">
@@ -45870,27 +45870,27 @@
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>MERCENARY</t>
+          <t>4F078</t>
         </is>
       </c>
       <c r="T128" t="inlineStr">
         <is>
-          <t>4F078</t>
+          <t>4F079</t>
         </is>
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>4F079</t>
+          <t>4F07A</t>
         </is>
       </c>
       <c r="V128" t="inlineStr">
         <is>
-          <t>4F07A</t>
+          <t>4F002</t>
         </is>
       </c>
       <c r="W128" t="inlineStr">
         <is>
-          <t>4F002</t>
+          <t>40008</t>
         </is>
       </c>
       <c r="X128" t="inlineStr">
@@ -46076,7 +46076,7 @@
       </c>
       <c r="CC128" t="inlineStr">
         <is>
-          <t>40008</t>
+          <t>ipbde03</t>
         </is>
       </c>
       <c r="CD128" t="n">
@@ -46084,7 +46084,7 @@
       </c>
       <c r="CE128" t="inlineStr">
         <is>
-          <t>ipbde03</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF128" t="n">
@@ -46212,7 +46212,7 @@
       <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -46567,7 +46567,7 @@
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
@@ -46922,7 +46922,7 @@
       <c r="O131" t="inlineStr"/>
       <c r="P131" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
@@ -47277,7 +47277,7 @@
       <c r="O132" t="inlineStr"/>
       <c r="P132" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
@@ -47632,7 +47632,7 @@
       <c r="O133" t="inlineStr"/>
       <c r="P133" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
@@ -47987,7 +47987,7 @@
       <c r="O134" t="inlineStr"/>
       <c r="P134" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -48342,7 +48342,7 @@
       <c r="O135" t="inlineStr"/>
       <c r="P135" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -48697,7 +48697,7 @@
       <c r="O136" t="inlineStr"/>
       <c r="P136" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -49052,7 +49052,7 @@
       <c r="O137" t="inlineStr"/>
       <c r="P137" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖАь»з</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -49407,12 +49407,12 @@
       <c r="O138" t="inlineStr"/>
       <c r="P138" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>巡察队</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>Стрелок</t>
+          <t>RANGER</t>
         </is>
       </c>
       <c r="R138" t="n">
@@ -49420,7 +49420,7 @@
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>RANGER</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -49626,7 +49626,7 @@
       </c>
       <c r="CC138" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqaaa00</t>
         </is>
       </c>
       <c r="CD138" t="n">
@@ -49634,7 +49634,7 @@
       </c>
       <c r="CE138" t="inlineStr">
         <is>
-          <t>iqaaa00</t>
+          <t>ipahp00</t>
         </is>
       </c>
       <c r="CF138" t="n">
@@ -49642,7 +49642,7 @@
       </c>
       <c r="CG138" t="inlineStr">
         <is>
-          <t>ipahp00</t>
+          <t>ipafp00</t>
         </is>
       </c>
       <c r="CH138" t="n">
@@ -49762,12 +49762,12 @@
       <c r="O139" t="inlineStr"/>
       <c r="P139" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>砲兵</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>Канонир</t>
+          <t>GUNNER</t>
         </is>
       </c>
       <c r="R139" t="n">
@@ -49775,22 +49775,22 @@
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>GUNNER</t>
+          <t>4F0EA</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
         <is>
-          <t>4F0EA</t>
+          <t>410EB</t>
         </is>
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>410EB</t>
+          <t>410EC</t>
         </is>
       </c>
       <c r="V139" t="inlineStr">
         <is>
-          <t>410EC</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W139" t="inlineStr">
@@ -49981,7 +49981,7 @@
       </c>
       <c r="CC139" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwlub30</t>
         </is>
       </c>
       <c r="CD139" t="n">
@@ -49989,7 +49989,7 @@
       </c>
       <c r="CE139" t="inlineStr">
         <is>
-          <t>iwlub30</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="CF139" t="n">
@@ -50117,12 +50117,12 @@
       <c r="O140" t="inlineStr"/>
       <c r="P140" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>侦察员</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>Лазутчик</t>
+          <t>SCOUTER</t>
         </is>
       </c>
       <c r="R140" t="n">
@@ -50130,22 +50130,22 @@
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>SCOUTER</t>
+          <t>4F0ED</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
         <is>
-          <t>4F0ED</t>
+          <t>4F0EE</t>
         </is>
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>4F0EE</t>
+          <t>4F0EF</t>
         </is>
       </c>
       <c r="V140" t="inlineStr">
         <is>
-          <t>4F0EF</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W140" t="inlineStr">
@@ -50336,7 +50336,7 @@
       </c>
       <c r="CC140" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwfib30</t>
         </is>
       </c>
       <c r="CD140" t="n">
@@ -50344,7 +50344,7 @@
       </c>
       <c r="CE140" t="inlineStr">
         <is>
-          <t>iwfib30</t>
+          <t>tr00001</t>
         </is>
       </c>
       <c r="CF140" t="n">
@@ -50472,12 +50472,12 @@
       <c r="O141" t="inlineStr"/>
       <c r="P141" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>天威炮将</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>Ракетчик</t>
+          <t>STRIKER</t>
         </is>
       </c>
       <c r="R141" t="n">
@@ -50485,22 +50485,22 @@
       </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>STRIKER</t>
+          <t>410ED</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
         <is>
-          <t>410ED</t>
+          <t>410EF</t>
         </is>
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>410EF</t>
+          <t>4F0F1</t>
         </is>
       </c>
       <c r="V141" t="inlineStr">
         <is>
-          <t>4F0F1</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W141" t="inlineStr">
@@ -50691,7 +50691,7 @@
       </c>
       <c r="CC141" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ibfir40</t>
         </is>
       </c>
       <c r="CD141" t="n">
@@ -50699,7 +50699,7 @@
       </c>
       <c r="CE141" t="inlineStr">
         <is>
-          <t>ibfir40</t>
+          <t>ibfir41</t>
         </is>
       </c>
       <c r="CF141" t="n">
@@ -50707,7 +50707,7 @@
       </c>
       <c r="CG141" t="inlineStr">
         <is>
-          <t>ibfir41</t>
+          <t>ibfir42</t>
         </is>
       </c>
       <c r="CH141" t="n">
@@ -50827,12 +50827,12 @@
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>暴走战狂</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>Дементер</t>
+          <t>DEMENTER</t>
         </is>
       </c>
       <c r="R142" t="n">
@@ -50840,27 +50840,27 @@
       </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>DEMENTER</t>
+          <t>4F0F3</t>
         </is>
       </c>
       <c r="T142" t="inlineStr">
         <is>
-          <t>4F0F3</t>
+          <t>4F0FA</t>
         </is>
       </c>
       <c r="U142" t="inlineStr">
         <is>
-          <t>4F0FA</t>
+          <t>4F0F5</t>
         </is>
       </c>
       <c r="V142" t="inlineStr">
         <is>
-          <t>4F0F5</t>
+          <t>4100C</t>
         </is>
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>4100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="X142" t="inlineStr">
@@ -51046,7 +51046,7 @@
       </c>
       <c r="CC142" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>ibbow48</t>
         </is>
       </c>
       <c r="CD142" t="n">
@@ -51054,7 +51054,7 @@
       </c>
       <c r="CE142" t="inlineStr">
         <is>
-          <t>ibbow48</t>
+          <t>ibfir34</t>
         </is>
       </c>
       <c r="CF142" t="n">
@@ -51062,7 +51062,7 @@
       </c>
       <c r="CG142" t="inlineStr">
         <is>
-          <t>ibfir34</t>
+          <t>ibfir36</t>
         </is>
       </c>
       <c r="CH142" t="n">
@@ -51182,12 +51182,12 @@
       <c r="O143" t="inlineStr"/>
       <c r="P143" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>幻影神兵</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>Фантом</t>
+          <t>PHANTOMSHADOW</t>
         </is>
       </c>
       <c r="R143" t="n">
@@ -51195,22 +51195,22 @@
       </c>
       <c r="S143" t="inlineStr">
         <is>
-          <t>PHANTOMSHADOW</t>
+          <t>400F6</t>
         </is>
       </c>
       <c r="T143" t="inlineStr">
         <is>
-          <t>400F6</t>
+          <t>4F0F7</t>
         </is>
       </c>
       <c r="U143" t="inlineStr">
         <is>
-          <t>4F0F7</t>
+          <t>4100C</t>
         </is>
       </c>
       <c r="V143" t="inlineStr">
         <is>
-          <t>4100C</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W143" t="inlineStr">
@@ -51401,7 +51401,7 @@
       </c>
       <c r="CC143" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iwdka40</t>
         </is>
       </c>
       <c r="CD143" t="n">
@@ -51409,7 +51409,7 @@
       </c>
       <c r="CE143" t="inlineStr">
         <is>
-          <t>iwdka40</t>
+          <t>tr00002</t>
         </is>
       </c>
       <c r="CF143" t="n">
@@ -51537,7 +51537,7 @@
       <c r="O144" t="inlineStr"/>
       <c r="P144" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q144" t="inlineStr">
@@ -51892,7 +51892,7 @@
       <c r="O145" t="inlineStr"/>
       <c r="P145" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q145" t="inlineStr">
@@ -52247,7 +52247,7 @@
       <c r="O146" t="inlineStr"/>
       <c r="P146" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
@@ -52602,7 +52602,7 @@
       <c r="O147" t="inlineStr"/>
       <c r="P147" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
@@ -52957,7 +52957,7 @@
       <c r="O148" t="inlineStr"/>
       <c r="P148" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr">
@@ -53312,7 +53312,7 @@
       <c r="O149" t="inlineStr"/>
       <c r="P149" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
@@ -53667,7 +53667,7 @@
       <c r="O150" t="inlineStr"/>
       <c r="P150" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q150" t="inlineStr">
@@ -54022,7 +54022,7 @@
       <c r="O151" t="inlineStr"/>
       <c r="P151" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q151" t="inlineStr">
@@ -54377,7 +54377,7 @@
       <c r="O152" t="inlineStr"/>
       <c r="P152" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖ·№АОАъ</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
@@ -54732,12 +54732,12 @@
       <c r="O153" t="inlineStr"/>
       <c r="P153" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>专家</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>Специалист</t>
+          <t>SPECIALIST</t>
         </is>
       </c>
       <c r="R153" t="n">
@@ -54745,7 +54745,7 @@
       </c>
       <c r="S153" t="inlineStr">
         <is>
-          <t>SPECIALIST</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="T153" t="inlineStr">
@@ -54951,7 +54951,7 @@
       </c>
       <c r="CC153" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iqaaa00</t>
         </is>
       </c>
       <c r="CD153" t="n">
@@ -54959,7 +54959,7 @@
       </c>
       <c r="CE153" t="inlineStr">
         <is>
-          <t>iqaaa00</t>
+          <t>iwmta00</t>
         </is>
       </c>
       <c r="CF153" t="n">
@@ -54967,7 +54967,7 @@
       </c>
       <c r="CG153" t="inlineStr">
         <is>
-          <t>iwmta00</t>
+          <t>itttt00</t>
         </is>
       </c>
       <c r="CH153" t="n">
@@ -55087,12 +55087,12 @@
       <c r="O154" t="inlineStr"/>
       <c r="P154" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>工程师</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>Инженер</t>
+          <t>ENGINEER</t>
         </is>
       </c>
       <c r="R154" t="n">
@@ -55100,12 +55100,12 @@
       </c>
       <c r="S154" t="inlineStr">
         <is>
-          <t>ENGINEER</t>
+          <t>4F1E6</t>
         </is>
       </c>
       <c r="T154" t="inlineStr">
         <is>
-          <t>4F1E6</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="U154" t="inlineStr">
@@ -55306,7 +55306,7 @@
       </c>
       <c r="CC154" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>gtaa001</t>
         </is>
       </c>
       <c r="CD154" t="n">
@@ -55442,7 +55442,7 @@
       <c r="O155" t="inlineStr"/>
       <c r="P155" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr">
@@ -55797,12 +55797,12 @@
       <c r="O156" t="inlineStr"/>
       <c r="P156" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>科学家</t>
         </is>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>Блок-Механик</t>
+          <t>SCIENTIST</t>
         </is>
       </c>
       <c r="R156" t="n">
@@ -55810,17 +55810,17 @@
       </c>
       <c r="S156" t="inlineStr">
         <is>
-          <t>SCIENTIST</t>
+          <t>4F1EC</t>
         </is>
       </c>
       <c r="T156" t="inlineStr">
         <is>
-          <t>4F1EC</t>
+          <t>4F1ED</t>
         </is>
       </c>
       <c r="U156" t="inlineStr">
         <is>
-          <t>4F1ED</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="V156" t="inlineStr">
@@ -56016,7 +56016,7 @@
       </c>
       <c r="CC156" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iaxxx09</t>
         </is>
       </c>
       <c r="CD156" t="n">
@@ -56024,7 +56024,7 @@
       </c>
       <c r="CE156" t="inlineStr">
         <is>
-          <t>iaxxx09</t>
+          <t>irgef03</t>
         </is>
       </c>
       <c r="CF156" t="n">
@@ -56032,7 +56032,7 @@
       </c>
       <c r="CG156" t="inlineStr">
         <is>
-          <t>irgef03</t>
+          <t>irgea03</t>
         </is>
       </c>
       <c r="CH156" t="n">
@@ -56152,12 +56152,12 @@
       <c r="O157" t="inlineStr"/>
       <c r="P157" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>战斗指挥</t>
         </is>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>Ведущий Звена</t>
+          <t>BATTLELEADER</t>
         </is>
       </c>
       <c r="R157" t="n">
@@ -56165,22 +56165,22 @@
       </c>
       <c r="S157" t="inlineStr">
         <is>
-          <t>BATTLELEADER</t>
+          <t>4F1EF</t>
         </is>
       </c>
       <c r="T157" t="inlineStr">
         <is>
-          <t>4F1EF</t>
+          <t>4F1F0</t>
         </is>
       </c>
       <c r="U157" t="inlineStr">
         <is>
-          <t>4F1F0</t>
+          <t>4F1F1</t>
         </is>
       </c>
       <c r="V157" t="inlineStr">
         <is>
-          <t>4F1F1</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="W157" t="inlineStr">
@@ -56371,7 +56371,7 @@
       </c>
       <c r="CC157" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>iaxxx09</t>
         </is>
       </c>
       <c r="CD157" t="n">
@@ -56379,7 +56379,7 @@
       </c>
       <c r="CE157" t="inlineStr">
         <is>
-          <t>iaxxx09</t>
+          <t>ibfir59</t>
         </is>
       </c>
       <c r="CF157" t="n">
@@ -56387,7 +56387,7 @@
       </c>
       <c r="CG157" t="inlineStr">
         <is>
-          <t>ibfir59</t>
+          <t>ibfir60</t>
         </is>
       </c>
       <c r="CH157" t="n">
@@ -56507,7 +56507,7 @@
       <c r="O158" t="inlineStr"/>
       <c r="P158" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr">
@@ -56862,7 +56862,7 @@
       <c r="O159" t="inlineStr"/>
       <c r="P159" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr">
@@ -57217,7 +57217,7 @@
       <c r="O160" t="inlineStr"/>
       <c r="P160" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr">
@@ -57572,7 +57572,7 @@
       <c r="O161" t="inlineStr"/>
       <c r="P161" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
@@ -57927,7 +57927,7 @@
       <c r="O162" t="inlineStr"/>
       <c r="P162" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr">
@@ -58282,7 +58282,7 @@
       <c r="O163" t="inlineStr"/>
       <c r="P163" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q163" t="inlineStr">
@@ -58637,7 +58637,7 @@
       <c r="O164" t="inlineStr"/>
       <c r="P164" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">
@@ -58992,7 +58992,7 @@
       <c r="O165" t="inlineStr"/>
       <c r="P165" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">
@@ -59347,7 +59347,7 @@
       <c r="O166" t="inlineStr"/>
       <c r="P166" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
@@ -59702,7 +59702,7 @@
       <c r="O167" t="inlineStr"/>
       <c r="P167" t="inlineStr">
         <is>
-          <t>ѕЖЕ©·№ЅГѕЖЖЇјц°и</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr">

</xml_diff>